<commit_message>
Alteração na manipulação do json e na escrita de informações dentro da planilha
</commit_message>
<xml_diff>
--- a/db/FARE26.xlsx
+++ b/db/FARE26.xlsx
@@ -10,14 +10,14 @@
     <sheet sheetId="1" name="FARE26" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Database">FARE26!$A$1:$V$14</definedName>
+    <definedName name="_xlnm.Database">FARE26!$A$1:$U$14</definedName>
   </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="100">
   <si>
     <t>DATA</t>
   </si>
@@ -31,9 +31,6 @@
     <t>ANO</t>
   </si>
   <si>
-    <t>SP_POA</t>
-  </si>
-  <si>
     <t>SELLER</t>
   </si>
   <si>
@@ -317,6 +314,9 @@
   </si>
   <si>
     <t>teste 4</t>
+  </si>
+  <si>
+    <t>23/10/2026</t>
   </si>
 </sst>
 </file>
@@ -675,24 +675,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:V17"/>
+  <dimension ref="A1:U18"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.77734375" customWidth="1"/>
     <col min="2" max="2" width="7.77734375" style="1" customWidth="1"/>
     <col min="3" max="3" width="4.77734375" style="1" customWidth="1"/>
     <col min="4" max="4" width="2.77734375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="1.77734375" style="1" customWidth="1"/>
-    <col min="6" max="7" width="20.77734375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" style="2" customWidth="1"/>
-    <col min="9" max="9" width="14.77734375" style="3" customWidth="1"/>
-    <col min="10" max="10" width="6.77734375" style="2" customWidth="1"/>
-    <col min="11" max="17" width="60.77734375" style="1" customWidth="1"/>
-    <col min="18" max="21" width="8.77734375" customWidth="1"/>
-    <col min="22" max="22" width="11.77734375" style="1" customWidth="1"/>
+    <col min="5" max="6" width="20.77734375" style="1" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="14.77734375" style="3" customWidth="1"/>
+    <col min="9" max="9" width="6.77734375" style="2" customWidth="1"/>
+    <col min="10" max="16" width="60.77734375" style="1" customWidth="1"/>
+    <col min="17" max="20" width="8.77734375" customWidth="1"/>
+    <col min="21" max="21" width="11.77734375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -711,16 +710,16 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -741,7 +740,7 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
       <c r="R1" t="s">
@@ -753,40 +752,40 @@
       <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>46078</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>24</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="2">
+        <v>5000</v>
+      </c>
+      <c r="H2" s="3">
+        <v>1730</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J2" s="1" t="s">
         <v>26</v>
-      </c>
-      <c r="H2" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I2" s="3">
-        <v>1730</v>
-      </c>
-      <c r="J2" s="2">
-        <v>0.5</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>27</v>
@@ -794,110 +793,110 @@
       <c r="L2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="M2" s="1" t="s">
-        <v>29</v>
+      <c r="Q2" s="4">
+        <v>46143</v>
       </c>
       <c r="R2" s="4">
-        <v>46143</v>
+        <v>46173</v>
       </c>
       <c r="S2" s="4">
-        <v>46173</v>
+        <v>46184</v>
       </c>
       <c r="T2" s="4">
-        <v>46184</v>
-      </c>
-      <c r="U2" s="4">
         <v>46194</v>
       </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>46080</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="F3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G3" s="2">
+        <v>1988.52</v>
+      </c>
+      <c r="H3" s="3">
+        <v>1780</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1988.52</v>
-      </c>
-      <c r="I3" s="3">
-        <v>1780</v>
-      </c>
-      <c r="J3" s="2">
-        <v>0.5</v>
-      </c>
       <c r="K3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="L3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="M3" s="1" t="s">
+      <c r="N3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="O3" s="1" t="s">
-        <v>34</v>
+      <c r="Q3" s="4">
+        <v>46113</v>
       </c>
       <c r="R3" s="4">
-        <v>46113</v>
+        <v>46142</v>
       </c>
       <c r="S3" s="4">
-        <v>46142</v>
+        <v>46148</v>
       </c>
       <c r="T3" s="4">
-        <v>46148</v>
-      </c>
-      <c r="U3" s="4">
         <v>46158</v>
       </c>
-      <c r="V3" s="1" t="b">
+      <c r="U3" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>46080</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="2">
+        <v>1028.681</v>
+      </c>
+      <c r="H4" s="3">
+        <v>1710</v>
+      </c>
+      <c r="I4" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H4" s="2">
-        <v>1028.681</v>
-      </c>
-      <c r="I4" s="3">
-        <v>1710</v>
-      </c>
-      <c r="J4" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M4" s="1" t="s">
+      <c r="N4" s="1" t="s">
         <v>39</v>
       </c>
       <c r="O4" s="1" t="s">
@@ -906,57 +905,57 @@
       <c r="P4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="Q4" s="1" t="s">
-        <v>42</v>
+      <c r="Q4" s="4">
+        <v>46082</v>
       </c>
       <c r="R4" s="4">
         <v>46082</v>
       </c>
       <c r="S4" s="4">
-        <v>46082</v>
+        <v>46086</v>
       </c>
       <c r="T4" s="4">
-        <v>46086</v>
-      </c>
-      <c r="U4" s="4">
         <v>46096</v>
       </c>
-      <c r="V4" s="1" t="b">
+      <c r="U4" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" ht="14.4" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>46098</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="2">
+        <v>8000</v>
+      </c>
+      <c r="H5" s="3">
+        <v>1748.84</v>
+      </c>
+      <c r="I5" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="2">
-        <v>8000</v>
-      </c>
-      <c r="I5" s="3">
-        <v>1748.84</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="K5" s="1" t="s">
+      <c r="L5" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="N5" s="1" t="s">
         <v>47</v>
       </c>
       <c r="O5" s="1" t="s">
@@ -965,111 +964,111 @@
       <c r="P5" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="Q5" s="1" t="s">
-        <v>50</v>
+      <c r="Q5" s="4">
+        <v>46174</v>
       </c>
       <c r="R5" s="4">
-        <v>46174</v>
+        <v>46203</v>
       </c>
       <c r="S5" s="4">
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="T5" s="4">
-        <v>46205</v>
-      </c>
-      <c r="U5" s="4">
         <v>46214</v>
       </c>
-      <c r="V5" s="1" t="b">
+      <c r="U5" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>46098</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>43</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="H6" s="2">
+      <c r="G6" s="2">
         <v>8000</v>
       </c>
-      <c r="I6" s="3">
+      <c r="H6" s="3">
         <v>1810.35</v>
       </c>
-      <c r="J6" s="2">
+      <c r="I6" s="2">
         <v>0.5</v>
       </c>
-      <c r="K6" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="M6" s="1" t="s">
+      <c r="J6" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="N6" s="1" t="s">
         <v>47</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>48</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
+      </c>
+      <c r="Q6" s="4">
+        <v>46204</v>
       </c>
       <c r="R6" s="4">
-        <v>46204</v>
+        <v>46234</v>
       </c>
       <c r="S6" s="4">
-        <v>46234</v>
+        <v>46237</v>
       </c>
       <c r="T6" s="4">
-        <v>46237</v>
-      </c>
-      <c r="U6" s="4">
         <v>46247</v>
       </c>
-      <c r="V6" s="1" t="b">
+      <c r="U6" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>46119</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>54</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="2">
+        <v>4993.176</v>
+      </c>
+      <c r="H7" s="3">
+        <v>1780</v>
+      </c>
+      <c r="I7" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J7" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="H7" s="2">
-        <v>4993.176</v>
-      </c>
-      <c r="I7" s="3">
-        <v>1780</v>
-      </c>
-      <c r="J7" s="2">
-        <v>0.5</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>57</v>
@@ -1077,110 +1076,110 @@
       <c r="L7" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="N7" s="1" t="s">
         <v>59</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>61</v>
+      <c r="Q7" s="4">
+        <v>46143</v>
       </c>
       <c r="R7" s="4">
-        <v>46143</v>
+        <v>46173</v>
       </c>
       <c r="S7" s="4">
-        <v>46173</v>
+        <v>46175</v>
       </c>
       <c r="T7" s="4">
-        <v>46175</v>
-      </c>
-      <c r="U7" s="4">
         <v>46185</v>
       </c>
-      <c r="V7" s="1" t="b">
+      <c r="U7" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>46128</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" s="2">
+        <v>2000</v>
+      </c>
+      <c r="H8" s="3">
+        <v>1820</v>
+      </c>
+      <c r="I8" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="H8" s="2">
-        <v>2000</v>
-      </c>
-      <c r="I8" s="3">
-        <v>1820</v>
-      </c>
-      <c r="J8" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="K8" s="1" t="s">
+      <c r="L8" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="M8" s="1" t="s">
-        <v>66</v>
+      <c r="Q8" s="4">
+        <v>46128</v>
       </c>
       <c r="R8" s="4">
-        <v>46128</v>
+        <v>46152</v>
       </c>
       <c r="S8" s="4">
-        <v>46152</v>
+        <v>46156</v>
       </c>
       <c r="T8" s="4">
-        <v>46156</v>
-      </c>
-      <c r="U8" s="4">
         <v>46166</v>
       </c>
-      <c r="V8" s="1" t="b">
+      <c r="U8" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>46140</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="2">
+        <v>14997</v>
+      </c>
+      <c r="H9" s="3">
+        <v>1800</v>
+      </c>
+      <c r="I9" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J9" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="H9" s="2">
-        <v>14997</v>
-      </c>
-      <c r="I9" s="3">
-        <v>1800</v>
-      </c>
-      <c r="J9" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>69</v>
       </c>
       <c r="M9" s="1" t="s">
@@ -1195,52 +1194,52 @@
       <c r="P9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q9" s="1" t="s">
-        <v>74</v>
+      <c r="Q9" s="4">
+        <v>46204</v>
       </c>
       <c r="R9" s="4">
-        <v>46204</v>
+        <v>46234</v>
       </c>
       <c r="S9" s="4">
-        <v>46234</v>
+        <v>46240</v>
       </c>
       <c r="T9" s="4">
-        <v>46240</v>
-      </c>
-      <c r="U9" s="4">
         <v>46250</v>
       </c>
-      <c r="V9" s="1" t="b">
+      <c r="U9" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>46149</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G10" s="2">
+        <v>4982.821</v>
+      </c>
+      <c r="H10" s="3">
+        <v>1720</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J10" s="1" t="s">
         <v>75</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="H10" s="2">
-        <v>4982.821</v>
-      </c>
-      <c r="I10" s="3">
-        <v>1720</v>
-      </c>
-      <c r="J10" s="2">
-        <v>0.5</v>
       </c>
       <c r="K10" s="1" t="s">
         <v>76</v>
@@ -1248,111 +1247,111 @@
       <c r="L10" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="N10" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="O10" s="1" t="s">
-        <v>79</v>
+      <c r="Q10" s="4">
+        <v>46149</v>
       </c>
       <c r="R10" s="4">
-        <v>46149</v>
+        <v>46173</v>
       </c>
       <c r="S10" s="4">
-        <v>46173</v>
+        <v>46181</v>
       </c>
       <c r="T10" s="4">
-        <v>46181</v>
-      </c>
-      <c r="U10" s="4">
         <v>46191</v>
       </c>
-      <c r="V10" s="1" t="b">
+      <c r="U10" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>46185</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G11" s="2">
+        <v>8000</v>
+      </c>
+      <c r="H11" s="3">
+        <v>1750</v>
+      </c>
+      <c r="I11" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J11" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="H11" s="2">
-        <v>8000</v>
-      </c>
-      <c r="I11" s="3">
-        <v>1750</v>
-      </c>
-      <c r="J11" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="K11" s="1" t="s">
+      <c r="L11" s="1" t="s">
         <v>81</v>
       </c>
       <c r="M11" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="N11" s="1" t="s">
+      <c r="O11" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="P11" s="1" t="s">
-        <v>84</v>
+      <c r="Q11" s="4">
+        <v>46174</v>
       </c>
       <c r="R11" s="4">
-        <v>46174</v>
+        <v>46203</v>
       </c>
       <c r="S11" s="4">
-        <v>46203</v>
+        <v>46205</v>
       </c>
       <c r="T11" s="4">
-        <v>46205</v>
-      </c>
-      <c r="U11" s="4">
         <v>46215</v>
       </c>
-      <c r="V11" s="1" t="b">
+      <c r="U11" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>46205</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G12" s="2">
+        <v>998.63</v>
+      </c>
+      <c r="H12" s="3">
+        <v>1750</v>
+      </c>
+      <c r="I12" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J12" s="1" t="s">
         <v>85</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H12" s="2">
-        <v>998.63</v>
-      </c>
-      <c r="I12" s="3">
-        <v>1750</v>
-      </c>
-      <c r="J12" s="2">
-        <v>0.5</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>86</v>
@@ -1360,281 +1359,274 @@
       <c r="L12" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="M12" s="1" t="s">
+      <c r="N12" s="1" t="s">
         <v>88</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="P12" s="1" t="s">
-        <v>90</v>
+      <c r="Q12" s="4">
+        <v>46204</v>
       </c>
       <c r="R12" s="4">
-        <v>46204</v>
+        <v>46234</v>
       </c>
       <c r="S12" s="4">
-        <v>46234</v>
+        <v>46245</v>
       </c>
       <c r="T12" s="4">
-        <v>46245</v>
-      </c>
-      <c r="U12" s="4">
         <v>46255</v>
       </c>
-      <c r="V12" s="1" t="b">
+      <c r="U12" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>46210</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G13" s="2">
+        <v>998.64</v>
+      </c>
+      <c r="H13" s="3">
+        <v>1770</v>
+      </c>
+      <c r="I13" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J13" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H13" s="2">
-        <v>998.64</v>
-      </c>
-      <c r="I13" s="3">
-        <v>1770</v>
-      </c>
-      <c r="J13" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="K13" s="1" t="s">
+      <c r="L13" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="N13" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="M13" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>93</v>
+      <c r="Q13" s="4">
+        <v>46210</v>
       </c>
       <c r="R13" s="4">
-        <v>46210</v>
+        <v>46234</v>
       </c>
       <c r="S13" s="4">
-        <v>46234</v>
+        <v>46246</v>
       </c>
       <c r="T13" s="4">
-        <v>46246</v>
-      </c>
-      <c r="U13" s="4">
         <v>46256</v>
       </c>
-      <c r="V13" s="1" t="b">
+      <c r="U13" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>46248</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C14" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G14" s="2">
+        <v>5000</v>
+      </c>
+      <c r="H14" s="3">
+        <v>1890</v>
+      </c>
+      <c r="I14" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="J14" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="D14" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="H14" s="2">
-        <v>5000</v>
-      </c>
-      <c r="I14" s="3">
-        <v>1890</v>
-      </c>
-      <c r="J14" s="2">
-        <v>0.5</v>
-      </c>
-      <c r="K14" s="1" t="s">
+      <c r="L14" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="M14" s="1" t="s">
+      <c r="Q14" s="4">
+        <v>46266</v>
+      </c>
+      <c r="R14" s="4">
+        <v>46295</v>
+      </c>
+      <c r="S14" s="4">
+        <v>46301</v>
+      </c>
+      <c r="T14" s="4">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>96</v>
       </c>
-      <c r="R14" s="4">
-        <v>46266</v>
-      </c>
-      <c r="S14" s="4">
-        <v>46295</v>
-      </c>
-      <c r="T14" s="4">
-        <v>46301</v>
-      </c>
-      <c r="U14" s="4">
-        <v>46311</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>97</v>
-      </c>
       <c r="B15" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="L15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="M15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="N15" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="J16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="L16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="M16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="N16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>98</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="B17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F15" s="1" t="s">
+      <c r="C17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="D17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="E17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="F17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="J15" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="H17" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="I17" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="M15" s="1" t="s">
+      <c r="J17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="N15" s="1" t="s">
+      <c r="K17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="O15" s="1" t="s">
+      <c r="L17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="P15" s="1" t="s">
+      <c r="M17" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>97</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="D16" s="1" t="s">
+      <c r="N17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="O17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F16" s="1" t="s">
+      <c r="P17" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="K16" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="M16" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="N16" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>99</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="H17" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="K17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="L17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="M17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="N17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="O17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="P17" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q17" s="1" t="s">
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>99</v>
       </c>
     </row>

</xml_diff>